<commit_message>
Vrije opdracht: krona analyse uitgevoerd
</commit_message>
<xml_diff>
--- a/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
+++ b/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rache\Documents\dsfb2\dsfb2_workflows_portfolio\dsfb2_workflows_portfolio\projecten\2_vrije_opdracht\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{034E2E80-1EFB-4BB7-94B1-F4127B281AC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAFA7B5-FC52-4650-8719-B20B4B20BC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C104C96A-1DAA-47F4-991A-E00D7F69CD18}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Datum</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>kraken2 en bracken analyse uitgevoerd.</t>
+  </si>
+  <si>
+    <t>3 uur en 30 minuten</t>
   </si>
 </sst>
 </file>
@@ -667,7 +670,7 @@
         <v>17</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D9" s="10"/>
       <c r="F9" s="8"/>

</xml_diff>

<commit_message>
Vrije opdracht: Verder gewerkt aan krona analyse en prevalentie vergelijking, conclusie en discussie geschreven, README bijgewerkt
</commit_message>
<xml_diff>
--- a/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
+++ b/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rache\Documents\dsfb2\dsfb2_workflows_portfolio\dsfb2_workflows_portfolio\projecten\2_vrije_opdracht\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAFA7B5-FC52-4650-8719-B20B4B20BC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF95BA4-710B-4B17-9220-C364AFC0BE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C104C96A-1DAA-47F4-991A-E00D7F69CD18}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Datum</t>
   </si>
@@ -89,16 +89,25 @@
     <t>35 minuten</t>
   </si>
   <si>
-    <t>11 uur en 40 minuten</t>
-  </si>
-  <si>
     <t>Verder gewerkt aan krona analyse.</t>
   </si>
   <si>
     <t>kraken2 en bracken analyse uitgevoerd.</t>
   </si>
   <si>
-    <t>3 uur en 30 minuten</t>
+    <t>Verder gewerkt aan krona analyse, begin gemaakt aan relatieve prevalentie vergelijking.</t>
+  </si>
+  <si>
+    <t>4 uur en 35 minuten</t>
+  </si>
+  <si>
+    <t>16 uur 15 minuten</t>
+  </si>
+  <si>
+    <t>3 uur en 5 minuten</t>
+  </si>
+  <si>
+    <t>Verder gewerkt aan krona analyse en prevalentie vergelijking, conclusie en discussie geschreven</t>
   </si>
 </sst>
 </file>
@@ -185,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -207,11 +216,8 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -547,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46C6F99C-E1A4-41D6-82B9-496F38F35459}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" customWidth="1"/>
@@ -639,7 +645,7 @@
         <v>46141</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>14</v>
@@ -652,46 +658,84 @@
         <v>46148</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="5"/>
-      <c r="F8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="9">
+    </row>
+    <row r="9" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="7">
         <v>46150</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="10"/>
-      <c r="F9" s="8"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="10"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
+      <c r="D9" s="6"/>
+      <c r="F9" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="7">
+        <v>46151</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="F10" s="8">
+        <v>0.83333333333333337</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Vrije opdracht: Uitwerking stap 1 t/m 5 nagekeken.
</commit_message>
<xml_diff>
--- a/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
+++ b/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rache\Documents\dsfb2\dsfb2_workflows_portfolio\dsfb2_workflows_portfolio\projecten\2_vrije_opdracht\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF95BA4-710B-4B17-9220-C364AFC0BE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00537D87-201E-4697-A91E-234DD9253F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C104C96A-1DAA-47F4-991A-E00D7F69CD18}"/>
   </bookViews>
@@ -104,10 +104,10 @@
     <t>16 uur 15 minuten</t>
   </si>
   <si>
-    <t>3 uur en 5 minuten</t>
-  </si>
-  <si>
-    <t>Verder gewerkt aan krona analyse en prevalentie vergelijking, conclusie en discussie geschreven</t>
+    <t>4 uur en 30 minuten</t>
+  </si>
+  <si>
+    <t>Verder gewerkt aan krona analyse en prevalentie vergelijking, conclusie en discussie geschreven, README bijgewerkt, uitwerking stap 1 t/m 5 nagekeken.</t>
   </si>
 </sst>
 </file>
@@ -680,7 +680,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
         <v>46151</v>
       </c>
@@ -692,7 +692,7 @@
       </c>
       <c r="D10" s="6"/>
       <c r="F10" s="8">
-        <v>0.83333333333333337</v>
+        <v>0.90555555555555556</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Opdracht 2. Vrije opdracht afgerond
</commit_message>
<xml_diff>
--- a/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
+++ b/projecten/2_vrije_opdracht/logboek_vrije_opdracht.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rache\Documents\dsfb2\dsfb2_workflows_portfolio\dsfb2_workflows_portfolio\projecten\2_vrije_opdracht\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00537D87-201E-4697-A91E-234DD9253F46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE1B0F3-3D59-4276-AA6A-82F5BFFE9FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C104C96A-1DAA-47F4-991A-E00D7F69CD18}"/>
+    <workbookView xWindow="0" yWindow="50" windowWidth="19200" windowHeight="10030" xr2:uid="{C104C96A-1DAA-47F4-991A-E00D7F69CD18}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>Datum</t>
   </si>
@@ -101,13 +101,41 @@
     <t>4 uur en 35 minuten</t>
   </si>
   <si>
-    <t>16 uur 15 minuten</t>
+    <t>Verder gewerkt aan krona analyse en prevalentie vergelijking, conclusie en discussie geschreven, README bijgewerkt, uitwerking stap 1 t/m 5 nagekeken.</t>
+  </si>
+  <si>
+    <t>5 uur</t>
+  </si>
+  <si>
+    <t>Uitwerking stap 6 t/m 10 nagekeken, kraken2 
+en bracken bestanden in repository geplaatst, README bijgewerkt.</t>
+  </si>
+  <si>
+    <t>link naar vorige opdracht</t>
   </si>
   <si>
     <t>4 uur en 30 minuten</t>
   </si>
   <si>
-    <t>Verder gewerkt aan krona analyse en prevalentie vergelijking, conclusie en discussie geschreven, README bijgewerkt, uitwerking stap 1 t/m 5 nagekeken.</t>
+    <t>Alles in bookdown zetten</t>
+  </si>
+  <si>
+    <t>3 uur en 15 minuten</t>
+  </si>
+  <si>
+    <t>reader goed bekijken of alles klopt!</t>
+  </si>
+  <si>
+    <t>1 uur</t>
+  </si>
+  <si>
+    <t>30 uur</t>
+  </si>
+  <si>
+    <t>Layout verslag bijgewerkt.</t>
+  </si>
+  <si>
+    <t>Bestand in bookdown gezet.</t>
   </si>
 </sst>
 </file>
@@ -194,7 +222,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -217,6 +245,12 @@
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -676,64 +710,88 @@
         <v>19</v>
       </c>
       <c r="D9" s="6"/>
-      <c r="F9" s="9" t="s">
-        <v>20</v>
-      </c>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
         <v>46151</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="F10" s="8">
-        <v>0.90555555555555556</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
+      <c r="F10" s="10"/>
+    </row>
+    <row r="11" spans="1:6" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A11" s="7">
+        <v>46152</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="D11" s="6"/>
+      <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
+      <c r="A12" s="7">
+        <v>46153</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>26</v>
+      </c>
       <c r="D12" s="6"/>
+      <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
+      <c r="A13" s="7">
+        <v>46155</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="11"/>
+      <c r="F13" s="8" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
+      <c r="B15" s="9" t="s">
+        <v>25</v>
+      </c>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
+      <c r="B16" s="9" t="s">
+        <v>23</v>
+      </c>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
+      <c r="B17" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
     </row>

</xml_diff>